<commit_message>
[Item Data] UseItemType 및 UseItemparameter 필드 추가와 Item_DummyBox_1 데이터 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Item.xlsx
+++ b/JsonConverter/ExcelFiles/Item.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6720"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="30468" windowHeight="12840"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,90 +19,117 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+  <x:si>
+    <x:t>StatChangeHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseItemType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Normal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토 주스</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
   <x:si>
     <x:t>당근 스무디</x:t>
   </x:si>
   <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Epic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RandomItemBox의 파라미터는 획득할 수 있는 아이템 Id 리스트
+StartChangeAtk의 파라미터는 음수 양수로 ATK 버프 디버프
+StartChangeHp의 파라미터는 음수 양수로 HP 버프 디버프
+SummonMonster의 파라미터는 소환할 수 있는 몬스터의 Id 리스트</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_CarrotSmoothy_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_Potion_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>물약</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>잘 익은 토마토를 담은 새콤한 주스 (HP +70)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_CarrotSmoothy_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>신선한 당근을 갈아 만든 건강 스무디 (HP + 50)</x:t>
   </x:si>
   <x:si>
-    <x:t>잘 익은 토마토를 담은 새콤한 주스 (HP +70)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Heal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>물약</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Potion_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_TomatoJuice_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grade</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Normal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토마토 주스</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ItemType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
+    <x:t>Icon/Icon_Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>체력을 회복시켜주는 기본 물약 (HP +30)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Potion_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
   </x:si>
   <x:si>
     <x:t>MaxStackCount</x:t>
   </x:si>
   <x:si>
-    <x:t>Item_Potion_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_CarrotSmoothy_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>체력을 회복시켜주는 기본 물약 (HP +30)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_TomatoJuice_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_CarrotSmoothy_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Epic</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Rare</x:t>
+    <x:t>랜덤 상자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseItemparameter</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RandomItemBox</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Potion_1:2,Item_CarrotSmoothy_1:1,Item_TomatoJuice_1:1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -273,8 +300,8 @@
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -880,178 +907,213 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:M35"/>
+  <x:dimension ref="A1:N35"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="21.33203125" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="42" style="2" customWidth="1"/>
-    <x:col min="4" max="4" width="10.66796875" style="2" customWidth="1"/>
-    <x:col min="5" max="5" width="12.5703125" style="2"/>
-    <x:col min="6" max="6" width="14.109375" style="2" customWidth="1"/>
-    <x:col min="7" max="8" width="43.109375" style="2" customWidth="1"/>
-    <x:col min="9" max="16384" width="12.5703125" style="2"/>
+    <x:col min="4" max="4" width="12.5703125" style="2"/>
+    <x:col min="5" max="5" width="14.109375" style="2" customWidth="1"/>
+    <x:col min="6" max="6" width="43.109375" style="2" customWidth="1"/>
+    <x:col min="7" max="7" width="14.4453125" style="2" customWidth="1"/>
+    <x:col min="8" max="8" width="55.22265625" style="2" customWidth="1"/>
+    <x:col min="9" max="9" width="43.109375" style="2" customWidth="1"/>
+    <x:col min="10" max="16384" width="12.5703125" style="2"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:8" ht="115.8" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:8" ht="13.199999999999999">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H1" s="14" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I2" s="1"/>
+    </x:row>
+    <x:row r="3" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="11" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D3" s="13" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="H2" s="1"/>
-    </x:row>
-    <x:row r="3" spans="1:8" s="12" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="11" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="s">
+      <x:c r="E3" s="13" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C3" s="11" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="D3" s="14" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E3" s="13" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F3" s="13" t="s">
-        <x:v>19</x:v>
-      </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H3" s="13"/>
-    </x:row>
-    <x:row r="4" spans="1:13" ht="15.75" customHeight="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H3" s="13" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="I3" s="13"/>
+    </x:row>
+    <x:row r="4" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F4" s="4">
+      <x:c r="E4" s="4">
         <x:v>10</x:v>
       </x:c>
+      <x:c r="F4" s="4" t="s">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="G4" s="4" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H4" s="4"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="4">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
       <x:c r="K4" s="4"/>
       <x:c r="L4" s="4"/>
       <x:c r="M4" s="4"/>
-    </x:row>
-    <x:row r="5" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N4" s="4"/>
+    </x:row>
+    <x:row r="5" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>22</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E5" s="4">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="F5" s="4">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="H5" s="4"/>
+      <x:c r="H5" s="4">
+        <x:v>50</x:v>
+      </x:c>
       <x:c r="I5" s="4"/>
-      <x:c r="K5" s="4"/>
+      <x:c r="J5" s="4"/>
       <x:c r="L5" s="4"/>
       <x:c r="M5" s="4"/>
-    </x:row>
-    <x:row r="6" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N5" s="4"/>
+    </x:row>
+    <x:row r="6" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>2</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E6" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E6" s="4" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F6" s="4">
-        <x:v>3</x:v>
+      <x:c r="F6" s="4" t="s">
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G6" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="H6" s="4"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="4">
+        <x:v>70</x:v>
+      </x:c>
       <x:c r="I6" s="4"/>
       <x:c r="J6" s="4"/>
       <x:c r="K6" s="4"/>
       <x:c r="L6" s="4"/>
       <x:c r="M6" s="4"/>
-    </x:row>
-    <x:row r="7" spans="1:13" ht="15.75" customHeight="1">
-      <x:c r="A7" s="3"/>
-      <x:c r="B7" s="5"/>
+      <x:c r="N6" s="4"/>
+    </x:row>
+    <x:row r="7" spans="1:14" ht="15.75" customHeight="1">
+      <x:c r="A7" s="3" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
+        <x:v>31</x:v>
+      </x:c>
       <x:c r="C7" s="5"/>
-      <x:c r="D7" s="4"/>
-      <x:c r="E7" s="4"/>
-      <x:c r="F7" s="4"/>
-      <x:c r="G7" s="4"/>
-      <x:c r="H7" s="4"/>
+      <x:c r="D7" s="4" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E7" s="4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
       <x:c r="K7" s="4"/>
       <x:c r="L7" s="4"/>
       <x:c r="M7" s="4"/>
-    </x:row>
-    <x:row r="8" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N7" s="4"/>
+    </x:row>
+    <x:row r="8" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A8" s="3"/>
       <x:c r="B8" s="3"/>
       <x:c r="C8" s="3"/>
@@ -1065,8 +1127,9 @@
       <x:c r="K8" s="4"/>
       <x:c r="L8" s="4"/>
       <x:c r="M8" s="4"/>
-    </x:row>
-    <x:row r="9" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N8" s="4"/>
+    </x:row>
+    <x:row r="9" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A9" s="6"/>
       <x:c r="B9" s="6"/>
       <x:c r="C9" s="6"/>
@@ -1080,8 +1143,9 @@
       <x:c r="K9" s="4"/>
       <x:c r="L9" s="4"/>
       <x:c r="M9" s="4"/>
-    </x:row>
-    <x:row r="10" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N9" s="4"/>
+    </x:row>
+    <x:row r="10" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A10" s="1"/>
       <x:c r="B10" s="1"/>
       <x:c r="C10" s="1"/>
@@ -1095,8 +1159,9 @@
       <x:c r="K10" s="4"/>
       <x:c r="L10" s="4"/>
       <x:c r="M10" s="4"/>
-    </x:row>
-    <x:row r="11" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N10" s="4"/>
+    </x:row>
+    <x:row r="11" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A11" s="1"/>
       <x:c r="B11" s="1"/>
       <x:c r="C11" s="1"/>
@@ -1110,8 +1175,9 @@
       <x:c r="K11" s="4"/>
       <x:c r="L11" s="4"/>
       <x:c r="M11" s="4"/>
-    </x:row>
-    <x:row r="12" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N11" s="4"/>
+    </x:row>
+    <x:row r="12" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A12" s="6"/>
       <x:c r="B12" s="6"/>
       <x:c r="C12" s="6"/>
@@ -1125,8 +1191,9 @@
       <x:c r="K12" s="4"/>
       <x:c r="L12" s="4"/>
       <x:c r="M12" s="4"/>
-    </x:row>
-    <x:row r="13" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N12" s="4"/>
+    </x:row>
+    <x:row r="13" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A13" s="3"/>
       <x:c r="B13" s="3"/>
       <x:c r="C13" s="3"/>
@@ -1140,8 +1207,9 @@
       <x:c r="K13" s="4"/>
       <x:c r="L13" s="4"/>
       <x:c r="M13" s="4"/>
-    </x:row>
-    <x:row r="14" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N13" s="4"/>
+    </x:row>
+    <x:row r="14" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A14" s="1"/>
       <x:c r="B14" s="1"/>
       <x:c r="C14" s="1"/>
@@ -1155,8 +1223,9 @@
       <x:c r="K14" s="4"/>
       <x:c r="L14" s="4"/>
       <x:c r="M14" s="4"/>
-    </x:row>
-    <x:row r="15" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="N14" s="4"/>
+    </x:row>
+    <x:row r="15" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A15" s="1"/>
       <x:c r="B15" s="1"/>
       <x:c r="C15" s="1"/>
@@ -1170,6 +1239,7 @@
       <x:c r="K15" s="4"/>
       <x:c r="L15" s="4"/>
       <x:c r="M15" s="4"/>
+      <x:c r="N15" s="4"/>
     </x:row>
     <x:row r="16" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A16" s="7"/>

</xml_diff>

<commit_message>
[Fix - Item Data] 코인들 UseItemType 설정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Item.xlsx
+++ b/JsonConverter/ExcelFiles/Item.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6792"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="30468" windowHeight="12840"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,33 +19,75 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
+  <x:si>
+    <x:t>Icon/Icon_Item_GoldWellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>물약</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
   <x:si>
     <x:t>int</x:t>
   </x:si>
   <x:si>
-    <x:t>물약</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_CarrotSmoothy_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_WellbeingCoin_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>잘 익은 토마토를 담은 새콤한 주스 (HP +70)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_TomatoJuice_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>신선한 당근을 갈아 만든 건강 스무디 (HP + 50)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potion_1:2,Item_CarrotSmoothy_1:1,Item_TomatoJuice_1:1</x:t>
+    <x:t>Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>StatChangeHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxStackCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Potion_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>왕실에서 발행한 고급 화폐</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RandomItemBox</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토 주스</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙 코인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>당근 스무디</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>랜덤 상자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Epic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Normal</x:t>
   </x:si>
   <x:si>
     <x:t>RandomItemBox의 파라미터는 획득할 수 있는 아이템 Id 리스트
@@ -54,106 +96,67 @@
 SummonMonster의 파라미터는 소환할 수 있는 몬스터의 Id 리스트</x:t>
   </x:si>
   <x:si>
+    <x:t>Item_Potion_1:2,Item_CarrotSmoothy_1:1,Item_TomatoJuice_1:1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>황금 웰빙 코인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseItemType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
     <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
     <x:t>Description</x:t>
   </x:si>
   <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>황금 웰빙 코인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_GoldWellbeingCoin_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_TomatoJuice_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙 코인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>당근 스무디</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토마토 주스</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potion_1</x:t>
+    <x:t>Icon/Icon_Item_WellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>신선한 당근을 갈아 만든 건강 스무디 (HP + 50)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_CarrotSmoothy_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>잘 익은 토마토를 담은 새콤한 주스 (HP +70)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>체력을 회복시켜주는 기본 물약 (HP +30)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_GoldWellbeingCoin_1</x:t>
   </x:si>
   <x:si>
     <x:t>Item_CarrotSmoothy_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Rare</x:t>
-  </x:si>
-  <x:si>
-    <x:t>랜덤 상자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grade</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Epic</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Normal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UseItemType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string[]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>StatChangeHp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RandomItemBox</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_DummyBox_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>왕실에서 발행한 고급 화폐</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxStackCount</x:t>
+    <x:t>Item_WellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아국에서 널리 사용되는 기본 화폐</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Item_Potion_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Item_WellbeingCoin_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>UseItemParameterList</x:t>
   </x:si>
   <x:si>
-    <x:t>웰빙리아국에서 널리 사용되는 기본 화폐</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_DummyBox_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_GoldWellbeingCoin_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>체력을 회복시켜주는 기본 물약 (HP +30)</x:t>
+    <x:t>Currency</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -948,40 +951,40 @@
   <x:sheetData>
     <x:row r="1" spans="1:8" ht="115.8" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H1" s="14" t="s">
-        <x:v>9</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="I2" s="1"/>
     </x:row>
@@ -990,49 +993,49 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="11" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C3" s="11" t="s">
-        <x:v>11</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D3" s="13" t="s">
-        <x:v>26</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E3" s="13" t="s">
-        <x:v>36</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F3" s="13" t="s">
-        <x:v>12</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>29</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="I3" s="13"/>
     </x:row>
     <x:row r="4" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>22</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>43</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E4" s="4">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G4" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H4" s="4">
         <x:v>30</x:v>
@@ -1046,25 +1049,25 @@
     </x:row>
     <x:row r="5" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>23</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
         <x:v>18</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="4">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F5" s="4" t="s">
-        <x:v>3</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="G5" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H5" s="4">
         <x:v>50</x:v>
@@ -1077,25 +1080,25 @@
     </x:row>
     <x:row r="6" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>21</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>5</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E6" s="4">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="4" t="s">
-        <x:v>6</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G6" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H6" s="4">
         <x:v>70</x:v>
@@ -1109,26 +1112,26 @@
     </x:row>
     <x:row r="7" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>25</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C7" s="5"/>
       <x:c r="D7" s="4" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E7" s="4">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F7" s="4" t="s">
-        <x:v>41</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G7" s="4" t="s">
-        <x:v>33</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H7" s="4" t="s">
-        <x:v>8</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
@@ -1139,22 +1142,24 @@
     </x:row>
     <x:row r="8" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D8" s="4" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E8" s="4"/>
       <x:c r="F8" s="4" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G8" s="4"/>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="s">
+        <x:v>44</x:v>
+      </x:c>
       <x:c r="H8" s="4"/>
       <x:c r="I8" s="4"/>
       <x:c r="J8" s="4"/>
@@ -1165,22 +1170,24 @@
     </x:row>
     <x:row r="9" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>42</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>13</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>35</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D9" s="4" t="s">
-        <x:v>24</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E9" s="4"/>
       <x:c r="F9" s="4" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G9" s="4"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="s">
+        <x:v>44</x:v>
+      </x:c>
       <x:c r="H9" s="4"/>
       <x:c r="I9" s="4"/>
       <x:c r="J9" s="4"/>

</xml_diff>

<commit_message>
[Add - Item Data] GradeDataId 데이터 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Item.xlsx
+++ b/JsonConverter/ExcelFiles/Item.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="30468" windowHeight="12840"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="18828" windowHeight="6792"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,75 +19,87 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
+  <x:si>
+    <x:t xml:space="preserve"> </x:t>
+  </x:si>
+  <x:si>
+    <x:t>GradeDataId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>물약</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>황금 웰빙 코인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseItemType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Currency</x:t>
+  </x:si>
   <x:si>
     <x:t>Icon/Icon_Item_GoldWellbeingCoin_1</x:t>
   </x:si>
   <x:si>
-    <x:t>물약</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
+    <x:t>신선한 당근을 갈아 만든 건강 스무디 (HP + 50)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>잘 익은 토마토를 담은 새콤한 주스 (HP +70)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_WellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_CarrotSmoothy_1</x:t>
   </x:si>
   <x:si>
     <x:t>Item_TomatoJuice_1</x:t>
   </x:si>
   <x:si>
-    <x:t>StatChangeHp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxStackCount</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potion_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>왕실에서 발행한 고급 화폐</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RandomItemBox</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_DummyBox_1</x:t>
+    <x:t>웰빙 코인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>랜덤 상자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토 주스</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>당근 스무디</x:t>
   </x:si>
   <x:si>
     <x:t>string</x:t>
   </x:si>
   <x:si>
-    <x:t>토마토 주스</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙 코인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>당근 스무디</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Rare</x:t>
-  </x:si>
-  <x:si>
-    <x:t>랜덤 상자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Epic</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grade</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Normal</x:t>
+    <x:t>Item_Potion_1:2,Item_CarrotSmoothy_1:1,Item_TomatoJuice_1:1</x:t>
   </x:si>
   <x:si>
     <x:t>RandomItemBox의 파라미터는 획득할 수 있는 아이템 Id 리스트
@@ -96,67 +108,58 @@
 SummonMonster의 파라미터는 소환할 수 있는 몬스터의 Id 리스트</x:t>
   </x:si>
   <x:si>
-    <x:t>Item_Potion_1:2,Item_CarrotSmoothy_1:1,Item_TomatoJuice_1:1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>황금 웰빙 코인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string[]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UseItemType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_WellbeingCoin_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_TomatoJuice_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>신선한 당근을 갈아 만든 건강 스무디 (HP + 50)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_CarrotSmoothy_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>잘 익은 토마토를 담은 새콤한 주스 (HP +70)</x:t>
+    <x:t>Item_Potion_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>StatChangeHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxStackCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RandomItemBox</x:t>
+  </x:si>
+  <x:si>
+    <x:t>왕실에서 발행한 고급 화폐</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_DummyBox_1</x:t>
   </x:si>
   <x:si>
     <x:t>체력을 회복시켜주는 기본 물약 (HP +30)</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Item_DummyBox_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>Item_GoldWellbeingCoin_1</x:t>
   </x:si>
   <x:si>
     <x:t>Item_CarrotSmoothy_1</x:t>
   </x:si>
   <x:si>
+    <x:t>Icon/Icon_Item_Potion_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아국에서 널리 사용되는 기본 화폐</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseItemParameterList</x:t>
+  </x:si>
+  <x:si>
     <x:t>Item_WellbeingCoin_1</x:t>
   </x:si>
   <x:si>
-    <x:t>웰빙리아국에서 널리 사용되는 기본 화폐</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Potion_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UseItemParameterList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Currency</x:t>
+    <x:t>Grade_Rare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade_Epic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade_Normal</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -940,7 +943,7 @@
     <x:col min="1" max="1" width="24.4453125" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="42" style="2" customWidth="1"/>
-    <x:col min="4" max="4" width="12.5703125" style="2"/>
+    <x:col min="4" max="4" width="13.109375" style="2" customWidth="1"/>
     <x:col min="5" max="5" width="14.109375" style="2" customWidth="1"/>
     <x:col min="6" max="6" width="43.109375" style="2" customWidth="1"/>
     <x:col min="7" max="7" width="14.4453125" style="2" customWidth="1"/>
@@ -951,91 +954,91 @@
   <x:sheetData>
     <x:row r="1" spans="1:8" ht="115.8" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>29</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H1" s="14" t="s">
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I2" s="1"/>
     </x:row>
     <x:row r="3" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="11" t="s">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B3" s="11" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C3" s="11" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D3" s="13" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="13" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D3" s="13" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="E3" s="13" t="s">
-        <x:v>7</x:v>
-      </x:c>
       <x:c r="F3" s="13" t="s">
-        <x:v>28</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>27</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>43</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I3" s="13"/>
     </x:row>
     <x:row r="4" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
         <x:v>36</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
-        <x:v>22</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E4" s="4">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="4" t="s">
-        <x:v>42</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="G4" s="4" t="s">
-        <x:v>5</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="H4" s="4">
         <x:v>30</x:v>
@@ -1049,25 +1052,25 @@
     </x:row>
     <x:row r="5" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E5" s="4">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F5" s="4" t="s">
-        <x:v>34</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G5" s="4" t="s">
-        <x:v>5</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="H5" s="4">
         <x:v>50</x:v>
@@ -1080,25 +1083,25 @@
     </x:row>
     <x:row r="6" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>13</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
-        <x:v>20</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E6" s="4">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="4" t="s">
-        <x:v>32</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="4" t="s">
-        <x:v>5</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="H6" s="4">
         <x:v>70</x:v>
@@ -1112,26 +1115,26 @@
     </x:row>
     <x:row r="7" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>11</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C7" s="5"/>
       <x:c r="D7" s="4" t="s">
-        <x:v>22</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E7" s="4">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F7" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="G7" s="4" t="s">
-        <x:v>10</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H7" s="4" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
@@ -1142,23 +1145,23 @@
     </x:row>
     <x:row r="8" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
       <x:c r="D8" s="4" t="s">
-        <x:v>22</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E8" s="4"/>
       <x:c r="F8" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G8" s="4" t="s">
-        <x:v>44</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H8" s="4"/>
       <x:c r="I8" s="4"/>
@@ -1170,23 +1173,23 @@
     </x:row>
     <x:row r="9" spans="1:14" ht="15.75" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>25</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>9</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E9" s="4"/>
       <x:c r="F9" s="4" t="s">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G9" s="4" t="s">
-        <x:v>44</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H9" s="4"/>
       <x:c r="I9" s="4"/>
@@ -1204,7 +1207,9 @@
       <x:c r="E10" s="4"/>
       <x:c r="F10" s="4"/>
       <x:c r="G10" s="4"/>
-      <x:c r="H10" s="4"/>
+      <x:c r="H10" s="4" t="s">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I10" s="4"/>
       <x:c r="J10" s="4"/>
       <x:c r="K10" s="4"/>

</xml_diff>